<commit_message>
Feat: atualização da tabela custos do projeto
</commit_message>
<xml_diff>
--- a/Documentação/Cronograma_apex.xlsx
+++ b/Documentação/Cronograma_apex.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DTG-2025\Desktop\Apex\Documentação\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F74BF4C3-0CFB-4FB7-905F-CAE8456ECD87}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED8FD4CF-066A-4EED-9654-EBC42C1C82FD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8940" xr2:uid="{AFF5E02A-8DF2-48BF-AB92-38B432B4FE84}"/>
   </bookViews>
@@ -342,16 +342,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -363,10 +354,19 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2798,34 +2798,34 @@
       <c r="AA1" s="1"/>
     </row>
     <row r="2" spans="2:28" x14ac:dyDescent="0.3">
-      <c r="X2" s="17" t="s">
+      <c r="X2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="Y2" s="18"/>
-      <c r="Z2" s="18"/>
-      <c r="AA2" s="18"/>
+      <c r="Y2" s="25"/>
+      <c r="Z2" s="25"/>
+      <c r="AA2" s="25"/>
     </row>
     <row r="3" spans="2:28" x14ac:dyDescent="0.3">
-      <c r="X3" s="19" t="s">
+      <c r="X3" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="Y3" s="19" t="s">
+      <c r="Y3" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="Z3" s="19" t="s">
+      <c r="Z3" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="AA3" s="19" t="s">
+      <c r="AA3" s="17" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="2:28" x14ac:dyDescent="0.3">
-      <c r="X4" s="20" t="s">
+      <c r="X4" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="Y4" s="20"/>
-      <c r="Z4" s="20"/>
-      <c r="AA4" s="20"/>
+      <c r="Y4" s="21"/>
+      <c r="Z4" s="21"/>
+      <c r="AA4" s="21"/>
     </row>
     <row r="5" spans="2:28" x14ac:dyDescent="0.3">
       <c r="H5" s="7"/>
@@ -2905,12 +2905,12 @@
     </row>
     <row r="10" spans="2:28" x14ac:dyDescent="0.3">
       <c r="B10" s="11"/>
-      <c r="X10" s="21" t="s">
+      <c r="X10" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="Y10" s="22"/>
-      <c r="Z10" s="22"/>
-      <c r="AA10" s="23"/>
+      <c r="Y10" s="19"/>
+      <c r="Z10" s="19"/>
+      <c r="AA10" s="20"/>
       <c r="AB10" s="11"/>
     </row>
     <row r="11" spans="2:28" x14ac:dyDescent="0.3">
@@ -2956,12 +2956,12 @@
       </c>
     </row>
     <row r="14" spans="2:28" x14ac:dyDescent="0.3">
-      <c r="X14" s="20" t="s">
+      <c r="X14" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="Y14" s="24"/>
-      <c r="Z14" s="24"/>
-      <c r="AA14" s="25"/>
+      <c r="Y14" s="22"/>
+      <c r="Z14" s="22"/>
+      <c r="AA14" s="23"/>
     </row>
     <row r="15" spans="2:28" x14ac:dyDescent="0.3">
       <c r="X15" s="12" t="s">
@@ -2992,12 +2992,12 @@
       </c>
     </row>
     <row r="17" spans="24:27" x14ac:dyDescent="0.3">
-      <c r="X17" s="21" t="s">
+      <c r="X17" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="Y17" s="22"/>
-      <c r="Z17" s="22"/>
-      <c r="AA17" s="23"/>
+      <c r="Y17" s="19"/>
+      <c r="Z17" s="19"/>
+      <c r="AA17" s="20"/>
     </row>
     <row r="18" spans="24:27" x14ac:dyDescent="0.3">
       <c r="X18" s="13" t="s">

</xml_diff>